<commit_message>
Completed unit verification of scalar register
</commit_message>
<xml_diff>
--- a/verification test cases.xlsx
+++ b/verification test cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503E74F8E0CF3/Projects/New folder/MIPS-Processor/MIPS-Processor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90D2491B-F5F9-4DF7-A778-45047AB372E6}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94947A43-3E17-4CFC-8F6A-1AB35D23A3DC}"/>
   <bookViews>
-    <workbookView xWindow="35310" yWindow="2925" windowWidth="17355" windowHeight="11235" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
+    <workbookView xWindow="50310" yWindow="0" windowWidth="7395" windowHeight="15585" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Scalar Register" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>clk</t>
   </si>
@@ -69,6 +69,27 @@
   </si>
   <si>
     <t>Outputs</t>
+  </si>
+  <si>
+    <t>Cycle</t>
+  </si>
+  <si>
+    <t>Plan</t>
+  </si>
+  <si>
+    <t>Send 1 to 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> For 1 to 8 Send n to address n</t>
+  </si>
+  <si>
+    <t>Read 0 to 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read 10 </t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -443,60 +464,522 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEA7434-B280-4886-8577-F525C2568B51}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E14" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F14" t="s">
         <v>4</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G14" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H14" t="s">
         <v>6</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I14" t="s">
         <v>7</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J14" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>5</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>3</v>
+      </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20">
+        <v>2</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <v>5</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
+      </c>
+      <c r="I21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>8</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>6</v>
+      </c>
+      <c r="F22">
+        <v>6</v>
+      </c>
+      <c r="G22">
+        <v>5</v>
+      </c>
+      <c r="H22">
+        <v>4</v>
+      </c>
+      <c r="I22">
+        <v>4</v>
+      </c>
+      <c r="J22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>9</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>7</v>
+      </c>
+      <c r="F23">
+        <v>7</v>
+      </c>
+      <c r="G23">
+        <v>6</v>
+      </c>
+      <c r="H23">
+        <v>5</v>
+      </c>
+      <c r="I23">
+        <v>5</v>
+      </c>
+      <c r="J23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>10</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>8</v>
+      </c>
+      <c r="F24">
+        <v>8</v>
+      </c>
+      <c r="G24">
+        <v>7</v>
+      </c>
+      <c r="H24">
+        <v>6</v>
+      </c>
+      <c r="I24">
+        <v>6</v>
+      </c>
+      <c r="J24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>11</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>8</v>
+      </c>
+      <c r="H25">
+        <v>7</v>
+      </c>
+      <c r="I25">
+        <v>7</v>
+      </c>
+      <c r="J25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>12</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>8</v>
+      </c>
+      <c r="I26">
+        <v>8</v>
+      </c>
+      <c r="J26">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>13</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="J27">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>14</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>15</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>16</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>17</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>18</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>19</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>20</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>21</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>22</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>23</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="I13:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Completed RTL of busyboard
</commit_message>
<xml_diff>
--- a/verification test cases.xlsx
+++ b/verification test cases.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503E74F8E0CF3/Projects/New folder/MIPS-Processor/MIPS-Processor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94947A43-3E17-4CFC-8F6A-1AB35D23A3DC}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F75AC253-9B02-4E17-84D6-D5E6BD8E136B}"/>
   <bookViews>
-    <workbookView xWindow="50310" yWindow="0" windowWidth="7395" windowHeight="15585" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
+    <workbookView xWindow="30570" yWindow="1110" windowWidth="27000" windowHeight="14040" activeTab="1" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Scalar Register" sheetId="1" r:id="rId1"/>
+    <sheet name="Progress Tracker" sheetId="2" r:id="rId1"/>
+    <sheet name="Scalar Writeback" sheetId="3" r:id="rId2"/>
+    <sheet name="Scalar Register" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
   <si>
     <t>clk</t>
   </si>
@@ -90,14 +92,121 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Implementation</t>
+  </si>
+  <si>
+    <t>Verification</t>
+  </si>
+  <si>
+    <t>PHASE 1</t>
+  </si>
+  <si>
+    <t>Fetch</t>
+  </si>
+  <si>
+    <t>Decode</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Scalar Busyboard</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Scalar Registers</t>
+  </si>
+  <si>
+    <t>Scalar Writeback</t>
+  </si>
+  <si>
+    <t>Scalar ALU</t>
+  </si>
+  <si>
+    <t>Scalar ALU Queue</t>
+  </si>
+  <si>
+    <t>Scalar LSU</t>
+  </si>
+  <si>
+    <t>Scalar LSU Queue</t>
+  </si>
+  <si>
+    <t>DMEM</t>
+  </si>
+  <si>
+    <t>DMEM Arbiter</t>
+  </si>
+  <si>
+    <t>PHASE 2</t>
+  </si>
+  <si>
+    <t>Scalar MULDIV</t>
+  </si>
+  <si>
+    <t>Scalar MULDIV Queue</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Vector Registers</t>
+  </si>
+  <si>
+    <t>Vector Writeback</t>
+  </si>
+  <si>
+    <t>Vector Busyboard</t>
+  </si>
+  <si>
+    <t>Vector ALU</t>
+  </si>
+  <si>
+    <t>Vector ALU Queue</t>
+  </si>
+  <si>
+    <t>Vector LSU</t>
+  </si>
+  <si>
+    <t>Vector LSU queue</t>
+  </si>
+  <si>
+    <t>Phase 3</t>
+  </si>
+  <si>
+    <t>Vector MULDIV</t>
+  </si>
+  <si>
+    <t>Vector MULDIV queue</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>IMEM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -113,7 +222,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -121,21 +230,110 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF9999"/>
+      <color rgb="FFFFCC99"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -145,6 +343,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -463,6 +665,312 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E388C35-15D6-4EC3-9BCF-884033AD006A}">
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="41" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5">
+    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",B5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11">
+    <cfRule type="containsText" priority="5" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",F11)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",A1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",B3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7E7C31F-88E4-4C6E-B314-098BDBBBBEC1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEA7434-B280-4886-8577-F525C2568B51}">
   <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Refactored code and worked on architecture
</commit_message>
<xml_diff>
--- a/verification test cases.xlsx
+++ b/verification test cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503E74F8E0CF3/Projects/New folder/MIPS-Processor/MIPS-Processor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="166" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F75AC253-9B02-4E17-84D6-D5E6BD8E136B}"/>
+  <xr:revisionPtr revIDLastSave="170" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A84301DC-08D4-479C-98A9-F58CE8D79362}"/>
   <bookViews>
-    <workbookView xWindow="30570" yWindow="1110" windowWidth="27000" windowHeight="14040" activeTab="1" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
+    <workbookView xWindow="30345" yWindow="1095" windowWidth="27000" windowHeight="14040" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Tracker" sheetId="2" r:id="rId1"/>
@@ -249,27 +249,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -298,34 +304,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -343,10 +321,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -675,13 +649,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -693,145 +667,145 @@
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="C8" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="B14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="B15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>38</v>
       </c>
     </row>
@@ -843,118 +817,118 @@
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A16:C16"/>
   </mergeCells>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Pending">
+      <formula>NOT(ISERROR(SEARCH("Pending",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",A1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",B3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B5">
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="0" priority="6" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",B5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11">
     <cfRule type="containsText" priority="5" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",F11)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Pending">
-      <formula>NOT(ISERROR(SEARCH("Pending",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",A1)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",B3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1008,19 +982,19 @@
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1" t="s">
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J13" s="1"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" t="s">

</xml_diff>

<commit_message>
Complete implementation of RAT, Fixed a few issues and intergrations
</commit_message>
<xml_diff>
--- a/verification test cases.xlsx
+++ b/verification test cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503E74F8E0CF3/Projects/New folder/MIPS-Processor/MIPS-Processor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503e74f8e0cf3/Projects/RISCV-SIMD_Processor/RISCV-SIMD_Processor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="170" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A84301DC-08D4-479C-98A9-F58CE8D79362}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4040824E-6969-4BC6-8CA0-325A4373CC7A}"/>
   <bookViews>
-    <workbookView xWindow="30345" yWindow="1095" windowWidth="27000" windowHeight="14040" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Tracker" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
   <si>
     <t>clk</t>
   </si>
@@ -103,94 +103,82 @@
     <t>Verification</t>
   </si>
   <si>
-    <t>PHASE 1</t>
-  </si>
-  <si>
     <t>Fetch</t>
   </si>
   <si>
     <t>Decode</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Scalar Busyboard</t>
-  </si>
-  <si>
     <t>Complete</t>
   </si>
   <si>
-    <t>Scalar Registers</t>
-  </si>
-  <si>
-    <t>Scalar Writeback</t>
-  </si>
-  <si>
-    <t>Scalar ALU</t>
-  </si>
-  <si>
-    <t>Scalar ALU Queue</t>
-  </si>
-  <si>
-    <t>Scalar LSU</t>
-  </si>
-  <si>
-    <t>Scalar LSU Queue</t>
-  </si>
-  <si>
     <t>DMEM</t>
   </si>
   <si>
-    <t>DMEM Arbiter</t>
-  </si>
-  <si>
-    <t>PHASE 2</t>
-  </si>
-  <si>
-    <t>Scalar MULDIV</t>
-  </si>
-  <si>
-    <t>Scalar MULDIV Queue</t>
-  </si>
-  <si>
     <t>Pending</t>
   </si>
   <si>
     <t>Vector Registers</t>
   </si>
   <si>
-    <t>Vector Writeback</t>
-  </si>
-  <si>
-    <t>Vector Busyboard</t>
-  </si>
-  <si>
     <t>Vector ALU</t>
   </si>
   <si>
-    <t>Vector ALU Queue</t>
-  </si>
-  <si>
-    <t>Vector LSU</t>
-  </si>
-  <si>
-    <t>Vector LSU queue</t>
-  </si>
-  <si>
-    <t>Phase 3</t>
-  </si>
-  <si>
-    <t>Vector MULDIV</t>
-  </si>
-  <si>
-    <t>Vector MULDIV queue</t>
-  </si>
-  <si>
-    <t>Integration</t>
-  </si>
-  <si>
     <t>IMEM</t>
+  </si>
+  <si>
+    <t>instruction queues</t>
+  </si>
+  <si>
+    <t>Register Allocation table</t>
+  </si>
+  <si>
+    <t>Reorder Buffer</t>
+  </si>
+  <si>
+    <t>Scalar Register</t>
+  </si>
+  <si>
+    <t>Reservation Station</t>
+  </si>
+  <si>
+    <t>ALU</t>
+  </si>
+  <si>
+    <t>Writeback Arbitration</t>
+  </si>
+  <si>
+    <t>Operation bus</t>
+  </si>
+  <si>
+    <t>Common Data Bus</t>
+  </si>
+  <si>
+    <t>OOO Core</t>
+  </si>
+  <si>
+    <t>Core</t>
+  </si>
+  <si>
+    <t>Muldiv Unit</t>
+  </si>
+  <si>
+    <t>Loadstore unit</t>
+  </si>
+  <si>
+    <t>Instruction functionality</t>
+  </si>
+  <si>
+    <t>Memory</t>
+  </si>
+  <si>
+    <t>Branching</t>
+  </si>
+  <si>
+    <t>SIMD</t>
+  </si>
+  <si>
+    <t>in progress</t>
   </si>
 </sst>
 </file>
@@ -222,7 +210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -245,11 +233,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -262,6 +298,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -640,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E388C35-15D6-4EC3-9BCF-884033AD006A}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -661,174 +718,162 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>32</v>
+      <c r="A12" s="9" t="s">
+        <v>39</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="A13" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>38</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>38</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
+      <c r="A16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="A17" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="A18" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -839,73 +884,77 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
+      <c r="A22" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="15"/>
+      <c r="C22" s="16"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>36</v>
-      </c>
+      <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>47</v>
-      </c>
+      <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
     </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A18:C18"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1:XFD1048576">
+  <conditionalFormatting sqref="A14:XFD16 A13 D13:XFD13 A1:XFD12 A19:XFD21 D17:XFD18 A17 A23:XFD1048576 A22 D22:XFD22">
     <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Pending">
       <formula>NOT(ISERROR(SEARCH("Pending",A1)))</formula>
     </cfRule>
@@ -926,12 +975,13 @@
       <formula>NOT(ISERROR(SEARCH("In Progress",B5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F11">
+  <conditionalFormatting sqref="F12">
     <cfRule type="containsText" priority="5" operator="containsText" text="Complete">
-      <formula>NOT(ISERROR(SEARCH("Complete",F11)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Complete",F12)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Completed verification of operation bus interface
</commit_message>
<xml_diff>
--- a/verification test cases.xlsx
+++ b/verification test cases.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/773503e74f8e0cf3/Projects/RISCV-SIMD_Processor/RISCV-SIMD_Processor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4040824E-6969-4BC6-8CA0-325A4373CC7A}"/>
+  <xr:revisionPtr revIDLastSave="333" documentId="8_{10AD32D8-6992-4962-A6CD-AFE1B7339FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8CC8365-2ED7-4AF0-A2A5-5EBA40EAE3EF}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="9540" windowHeight="15585" activeTab="1" xr2:uid="{33D90C5A-8101-4503-8AC9-D985ED1294F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Progress Tracker" sheetId="2" r:id="rId1"/>
-    <sheet name="Scalar Writeback" sheetId="3" r:id="rId2"/>
-    <sheet name="Scalar Register" sheetId="1" r:id="rId3"/>
+    <sheet name="Operation Bus" sheetId="4" r:id="rId2"/>
+    <sheet name="Scalar Writeback" sheetId="3" r:id="rId3"/>
+    <sheet name="Scalar Register" sheetId="1" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
   <si>
     <t>clk</t>
   </si>
@@ -179,6 +180,30 @@
   </si>
   <si>
     <t>in progress</t>
+  </si>
+  <si>
+    <t>Checking if valid bit is being set correctly</t>
+  </si>
+  <si>
+    <t>rob_cs</t>
+  </si>
+  <si>
+    <t>rat_cs</t>
+  </si>
+  <si>
+    <t>reg_cs</t>
+  </si>
+  <si>
+    <t>rat_valid</t>
+  </si>
+  <si>
+    <t>rob_valid</t>
+  </si>
+  <si>
+    <t>reg_valid</t>
+  </si>
+  <si>
+    <t>occupied</t>
   </si>
 </sst>
 </file>
@@ -986,6 +1011,481 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F421C3D3-72A0-4C41-BA11-6F80FEDB1D01}">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>1</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>1</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>0</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>0</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>0</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>0</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7E7C31F-88E4-4C6E-B314-098BDBBBBEC1}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -994,7 +1494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEA7434-B280-4886-8577-F525C2568B51}">
   <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>